<commit_message>
revise: model audit fixes (net cash, event-selection bias, estimation window) + official 1-page cover
CRITICAL fix: net cash US$1.5bn -> US$0.55bn (net IPO proceeds + pre-IPO cash; preferred converts at IPO).
DCF per-share now HK$11/29/67, prob-weighted HK$30 (~1.5% of price). Excel + Appendix B + all docs synced.

Event study:
- event dates identified independently from official announcements (Fig 2 = descriptive cross-check only)
- add AR formula + [-20,-6] estimation window; recomputed CAR (avg react +18.7, drift +4.8)
- GLM-5.2 truncation marked in Tables 2 & 3 and Fig 3 (events 4->3 after +7); softened to preliminary PCAD

Other: reverse DCF '~105% annual over 2026-2035' (not ten-year CAGR); abstract Chapter-18C regime + earnings
wording; bottom-up beta rationale (short history); Feng Liu citation format fixed; title shortened.

Cover: rebuilt to official template (西南财经大学本科考试/课程论文, gray crest watermark, corner marks,
underlined fields), now a single page.
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -517,7 +517,12 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>1500</v>
+        <v>550</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>net IPO proceeds ~HK$4.3bn/7.8 + pre-IPO cash ~US$27m; preferred shares convert at IPO</t>
+        </is>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
fix: align valuation paper data and outputs
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -427,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -510,30 +511,47 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Market price (HK$)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2046</v>
+          <t>Market date</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>derived from data/Zhipu_KnowledgeAtlas_daily.csv</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025 revenue (US$m)</t>
+          <t>Market price (HK$)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>102</v>
+        <v>2046</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>2025 revenue (US$m)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>2026E revenue (US$m)</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B11" t="n">
         <v>200</v>
       </c>
     </row>
@@ -704,11 +722,11 @@
         <v>0</v>
       </c>
       <c r="C9">
-        <f>Assumptions!$B$10/Assumptions!$B$9-1</f>
+        <f>Assumptions!$B$11/Assumptions!$B$10-1</f>
         <v/>
       </c>
       <c r="D9">
-        <f>Assumptions!$B$10</f>
+        <f>Assumptions!$B$11</f>
         <v/>
       </c>
       <c r="E9">
@@ -732,7 +750,7 @@
         <v/>
       </c>
       <c r="J9">
-        <f>D9-Assumptions!$B$9</f>
+        <f>D9-Assumptions!$B$10</f>
         <v/>
       </c>
       <c r="K9">
@@ -1500,11 +1518,11 @@
         <v>0</v>
       </c>
       <c r="C9">
-        <f>Assumptions!$B$10/Assumptions!$B$9-1</f>
+        <f>Assumptions!$B$11/Assumptions!$B$10-1</f>
         <v/>
       </c>
       <c r="D9">
-        <f>Assumptions!$B$10</f>
+        <f>Assumptions!$B$11</f>
         <v/>
       </c>
       <c r="E9">
@@ -1528,7 +1546,7 @@
         <v/>
       </c>
       <c r="J9">
-        <f>D9-Assumptions!$B$9</f>
+        <f>D9-Assumptions!$B$10</f>
         <v/>
       </c>
       <c r="K9">
@@ -2296,11 +2314,11 @@
         <v>0</v>
       </c>
       <c r="C9">
-        <f>Assumptions!$B$10/Assumptions!$B$9-1</f>
+        <f>Assumptions!$B$11/Assumptions!$B$10-1</f>
         <v/>
       </c>
       <c r="D9">
-        <f>Assumptions!$B$10</f>
+        <f>Assumptions!$B$11</f>
         <v/>
       </c>
       <c r="E9">
@@ -2324,7 +2342,7 @@
         <v/>
       </c>
       <c r="J9">
-        <f>D9-Assumptions!$B$9</f>
+        <f>D9-Assumptions!$B$10</f>
         <v/>
       </c>
       <c r="K9">
@@ -3050,7 +3068,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>Assumptions!B8</f>
+        <f>Assumptions!B9</f>
         <v/>
       </c>
     </row>
@@ -3072,8 +3090,128 @@
         </is>
       </c>
       <c r="B9">
-        <f>(Assumptions!B8*Assumptions!B5/Assumptions!B6)/Assumptions!B10</f>
-        <v/>
+        <f>(Assumptions!B9*Assumptions!B5/Assumptions!B6)/Assumptions!B11</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Market date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Market price (HK$)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2046</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Market equity value (US$m)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>114103.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Market EV / FY2026E revenue</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>570.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Bear per share (HK$)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Base per share (HK$)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>28.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bull per share (HK$)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>81.59999999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Probability-weighted equity (US$m)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1853.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Probability-weighted per share (HK$)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>33.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DCF value as % of market</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.0162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: integrate AGM circular data and refresh Tushare prices
- Update shares outstanding from ~435M to 445.843M (AGM circular 2026-06-22)
- Add agm2513 bibliography entry and governance details (equity incentive
  scheme, issuance mandates, all 20 resolutions passed unanimously)
- Add AGM milestone to GLM timeline figure
- Refresh all 3 stock CSVs from Tushare (2026-06-30 still manual)
- Recascade all valuation outputs: mcap ~US$120B, EV/rev 601x,
  DCF base HK$27/share, prob-weighted HK$32 (1.5%), reverse DCF ~US$139B
- Update reverse-DCF sensitivity grid and heatmap with new market cap
- Sync README (CN/EN), DATA_TABLES.md, OUTLINE.md
- Fix validate_outputs word-count check to <= 3000 (matches ≤3000 spec)
- Update test expected per-share value from 28.1 to 27.4
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -480,7 +480,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>435</v>
+        <v>445.843</v>
       </c>
     </row>
     <row r="6">
@@ -516,7 +516,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2046</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="10">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2046</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="3">
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>114103.8</v>
+        <v>120263.3</v>
       </c>
     </row>
     <row r="4">
@@ -3151,7 +3151,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>570.5</v>
+        <v>601.3</v>
       </c>
     </row>
     <row r="5">
@@ -3161,7 +3161,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12.2</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="6">
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28.1</v>
+        <v>27.4</v>
       </c>
     </row>
     <row r="7">
@@ -3181,7 +3181,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>81.59999999999999</v>
+        <v>79.7</v>
       </c>
     </row>
     <row r="8">
@@ -3201,7 +3201,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>33.2</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="10">
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0162</v>
+        <v>0.0154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: refresh Zhipu market data to 2026-07-03
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2104</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="10">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2104</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="3">
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>120263.3</v>
+        <v>102486.7</v>
       </c>
     </row>
     <row r="4">
@@ -3151,7 +3151,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>601.3</v>
+        <v>512.4</v>
       </c>
     </row>
     <row r="5">
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0154</v>
+        <v>0.0181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: refresh core market data through 2026-07-10
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1793</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="10">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1793</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="3">
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>102486.7</v>
+        <v>93741.3</v>
       </c>
     </row>
     <row r="4">
@@ -3151,7 +3151,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>512.4</v>
+        <v>468.7</v>
       </c>
     </row>
     <row r="5">
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0181</v>
+        <v>0.0198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update paper and outputs to latest data
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1640</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="10">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1640</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="3">
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>93741.3</v>
+        <v>63275.4</v>
       </c>
     </row>
     <row r="4">
@@ -3151,7 +3151,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>468.7</v>
+        <v>316.4</v>
       </c>
     </row>
     <row r="5">
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0198</v>
+        <v>0.0293</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data to 2026-07-24 and regenerate outputs
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1107</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="10">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1107</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="3">
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>63275.4</v>
+        <v>70706.10000000001</v>
       </c>
     </row>
     <row r="4">
@@ -3151,7 +3151,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>316.4</v>
+        <v>353.5</v>
       </c>
     </row>
     <row r="5">
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0293</v>
+        <v>0.0262</v>
       </c>
     </row>
   </sheetData>

</xml_diff>